<commit_message>
Add Israeli schedule for Arab Israeli crews; fix scaling of authority durations in IL schedules
</commit_message>
<xml_diff>
--- a/05_תוצרים/לוח_זמנים_שלונסקי_53_ישראל_פועלים_סינים.xlsx
+++ b/05_תוצרים/לוח_זמנים_שלונסקי_53_ישראל_פועלים_סינים.xlsx
@@ -154,7 +154,7 @@
     <t>מקדם תפוקה:</t>
   </si>
   <si>
-    <t>משכי הבסיס מחושבים לימי עבודה של 8 שעות. המשך בפועל = משך הבסיס ÷ מקדם התפוקה (מעוגל כלפי מעלה). ב-10 שעות ביום המקדם 1.18 (תפוקה שולית יורדת). מגמת העבודה: א׳–ה׳. אפשר לשנות שעות, תאריך התחלה, משכים וחגים – התאריכים והגאנט מתעדכנים.</t>
+    <t>משכי הבסיס מחושבים לימי עבודה של 8 שעות. המשך בפועל = משך הבסיס ÷ מקדם התפוקה (מעוגל כלפי מעלה; משימות רשות/אישורים/ספקים/בדיקות קבועות אינן מוקטנות). ב-10 שעות ביום המקדם 1.18 (תפוקה שולית יורדת). מגמת העבודה: א׳–ה׳. אפשר לשנות שעות, תאריך התחלה, משכים וחגים – התאריכים והגאנט מתעדכנים.</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -2429,7 +2429,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="15">
-        <f>IF(D13=0,0,MAX(1,ROUNDUP(D13/$D$5,0)))</f>
+        <f>D13</f>
         <v>0</v>
       </c>
       <c r="F13" s="15" t="s">
@@ -2471,7 +2471,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="15">
-        <f>IF(D14=0,0,MAX(1,ROUNDUP(D14/$D$5,0)))</f>
+        <f>D14</f>
         <v>3</v>
       </c>
       <c r="F14" s="15" t="s">
@@ -2513,8 +2513,8 @@
         <v>10</v>
       </c>
       <c r="E15" s="15">
-        <f>IF(D15=0,0,MAX(1,ROUNDUP(D15/$D$5,0)))</f>
-        <v>9</v>
+        <f>D15</f>
+        <v>10</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>65</v>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="N15" s="18">
         <f>IF(E15=0,M15,WORKDAY.INTL(M15,E15-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="O15" s="19" t="s">
         <v>68</v>
@@ -2557,8 +2557,8 @@
         <v>40</v>
       </c>
       <c r="E16" s="15">
-        <f>IF(D16=0,0,MAX(1,ROUNDUP(D16/$D$5,0)))</f>
-        <v>34</v>
+        <f>D16</f>
+        <v>40</v>
       </c>
       <c r="F16" s="15" t="s">
         <v>65</v>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="N16" s="18">
         <f>IF(E16=0,M16,WORKDAY.INTL(M16,E16-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46380</v>
+        <v>46390</v>
       </c>
       <c r="O16" s="19"/>
       <c r="P16" s="15" t="s">
@@ -2599,8 +2599,8 @@
         <v>10</v>
       </c>
       <c r="E17" s="15">
-        <f>IF(D17=0,0,MAX(1,ROUNDUP(D17/$D$5,0)))</f>
-        <v>9</v>
+        <f>D17</f>
+        <v>10</v>
       </c>
       <c r="F17" s="15" t="s">
         <v>65</v>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="N17" s="18">
         <f>IF(E17=0,M17,WORKDAY.INTL(M17,E17-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="O17" s="19"/>
       <c r="P17" s="15" t="s">
@@ -2641,8 +2641,8 @@
         <v>20</v>
       </c>
       <c r="E18" s="15">
-        <f>IF(D18=0,0,MAX(1,ROUNDUP(D18/$D$5,0)))</f>
-        <v>17</v>
+        <f>D18</f>
+        <v>20</v>
       </c>
       <c r="F18" s="15" t="s">
         <v>82</v>
@@ -2654,15 +2654,15 @@
       <c r="K18" s="15"/>
       <c r="L18" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F18,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G18,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H18,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I18,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J18,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K18,$A$11:$A$86,0)),0))</f>
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="M18" s="18">
         <f>IF(E18=0,IF(COUNTA(F18:K18)=0,$D$2,L18),WORKDAY.INTL(L18,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N18" s="18">
         <f>IF(E18=0,M18,WORKDAY.INTL(M18,E18-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46370</v>
+        <v>46376</v>
       </c>
       <c r="O18" s="19"/>
       <c r="P18" s="15" t="s">
@@ -2683,8 +2683,8 @@
         <v>20</v>
       </c>
       <c r="E19" s="15">
-        <f>IF(D19=0,0,MAX(1,ROUNDUP(D19/$D$5,0)))</f>
-        <v>17</v>
+        <f>D19</f>
+        <v>20</v>
       </c>
       <c r="F19" s="15" t="s">
         <v>82</v>
@@ -2696,15 +2696,15 @@
       <c r="K19" s="15"/>
       <c r="L19" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F19,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G19,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H19,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I19,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J19,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K19,$A$11:$A$86,0)),0))</f>
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="M19" s="18">
         <f>IF(E19=0,IF(COUNTA(F19:K19)=0,$D$2,L19),WORKDAY.INTL(L19,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N19" s="18">
         <f>IF(E19=0,M19,WORKDAY.INTL(M19,E19-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46370</v>
+        <v>46376</v>
       </c>
       <c r="O19" s="19"/>
       <c r="P19" s="15" t="s">
@@ -2830,15 +2830,15 @@
       <c r="K21" s="15"/>
       <c r="L21" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F21,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G21,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H21,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I21,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J21,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K21,$A$11:$A$86,0)),0))</f>
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="M21" s="18">
         <f>IF(E21=0,IF(COUNTA(F21:K21)=0,$D$2,L21),WORKDAY.INTL(L21,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N21" s="18">
         <f>IF(E21=0,M21,WORKDAY.INTL(M21,E21-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46352</v>
+        <v>46355</v>
       </c>
       <c r="O21" s="19" t="s">
         <v>68</v>
@@ -2874,15 +2874,15 @@
       <c r="K22" s="15"/>
       <c r="L22" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F22,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G22,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H22,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I22,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J22,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K22,$A$11:$A$86,0)),0))</f>
-        <v>46352</v>
+        <v>46355</v>
       </c>
       <c r="M22" s="18">
         <f>IF(E22=0,IF(COUNTA(F22:K22)=0,$D$2,L22),WORKDAY.INTL(L22,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46355</v>
+        <v>46356</v>
       </c>
       <c r="N22" s="18">
         <f>IF(E22=0,M22,WORKDAY.INTL(M22,E22-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46358</v>
+        <v>46359</v>
       </c>
       <c r="O22" s="19" t="s">
         <v>68</v>
@@ -2905,7 +2905,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="15">
-        <f>IF(D23=0,0,MAX(1,ROUNDUP(D23/$D$5,0)))</f>
+        <f>D23</f>
         <v>1</v>
       </c>
       <c r="F23" s="15" t="s">
@@ -2918,15 +2918,15 @@
       <c r="K23" s="15"/>
       <c r="L23" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F23,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G23,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H23,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I23,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J23,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K23,$A$11:$A$86,0)),0))</f>
-        <v>46358</v>
+        <v>46359</v>
       </c>
       <c r="M23" s="18">
         <f>IF(E23=0,IF(COUNTA(F23:K23)=0,$D$2,L23),WORKDAY.INTL(L23,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="N23" s="18">
         <f>IF(E23=0,M23,WORKDAY.INTL(M23,E23-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="O23" s="19" t="s">
         <v>68</v>
@@ -3052,15 +3052,15 @@
       <c r="K25" s="15"/>
       <c r="L25" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F25,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G25,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H25,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I25,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J25,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K25,$A$11:$A$86,0)),0))</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="M25" s="18">
         <f>IF(E25=0,IF(COUNTA(F25:K25)=0,$D$2,L25),WORKDAY.INTL(L25,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46362</v>
+        <v>46363</v>
       </c>
       <c r="N25" s="18">
         <f>IF(E25=0,M25,WORKDAY.INTL(M25,E25-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="O25" s="19" t="s">
         <v>68</v>
@@ -3096,15 +3096,15 @@
       <c r="K26" s="15"/>
       <c r="L26" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F26,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G26,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H26,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I26,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J26,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K26,$A$11:$A$86,0)),0))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="M26" s="18">
         <f>IF(E26=0,IF(COUNTA(F26:K26)=0,$D$2,L26),WORKDAY.INTL(L26,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="N26" s="18">
         <f>IF(E26=0,M26,WORKDAY.INTL(M26,E26-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46373</v>
+        <v>46376</v>
       </c>
       <c r="O26" s="19"/>
       <c r="P26" s="15" t="s">
@@ -3138,15 +3138,15 @@
       <c r="K27" s="15"/>
       <c r="L27" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F27,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G27,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H27,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I27,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J27,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K27,$A$11:$A$86,0)),0))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="M27" s="18">
         <f>IF(E27=0,IF(COUNTA(F27:K27)=0,$D$2,L27),WORKDAY.INTL(L27,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="N27" s="18">
         <f>IF(E27=0,M27,WORKDAY.INTL(M27,E27-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46373</v>
+        <v>46376</v>
       </c>
       <c r="O27" s="19"/>
       <c r="P27" s="15" t="s">
@@ -3180,15 +3180,15 @@
       <c r="K28" s="15"/>
       <c r="L28" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F28,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G28,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H28,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I28,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J28,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K28,$A$11:$A$86,0)),0))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="M28" s="18">
         <f>IF(E28=0,IF(COUNTA(F28:K28)=0,$D$2,L28),WORKDAY.INTL(L28,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="N28" s="18">
         <f>IF(E28=0,M28,WORKDAY.INTL(M28,E28-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46376</v>
+        <v>46377</v>
       </c>
       <c r="O28" s="19"/>
       <c r="P28" s="15" t="s">
@@ -3222,15 +3222,15 @@
       <c r="K29" s="15"/>
       <c r="L29" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F29,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G29,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H29,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I29,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J29,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K29,$A$11:$A$86,0)),0))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="M29" s="18">
         <f>IF(E29=0,IF(COUNTA(F29:K29)=0,$D$2,L29),WORKDAY.INTL(L29,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="N29" s="18">
         <f>IF(E29=0,M29,WORKDAY.INTL(M29,E29-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="O29" s="19" t="s">
         <v>68</v>
@@ -3268,15 +3268,15 @@
       <c r="K30" s="15"/>
       <c r="L30" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F30,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G30,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H30,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I30,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J30,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K30,$A$11:$A$86,0)),0))</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="M30" s="18">
         <f>IF(E30=0,IF(COUNTA(F30:K30)=0,$D$2,L30),WORKDAY.INTL(L30,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46362</v>
+        <v>46363</v>
       </c>
       <c r="N30" s="18">
         <f>IF(E30=0,M30,WORKDAY.INTL(M30,E30-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46366</v>
+        <v>46369</v>
       </c>
       <c r="O30" s="19"/>
       <c r="P30" s="15" t="s">
@@ -3297,7 +3297,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="15">
-        <f>IF(D31=0,0,MAX(1,ROUNDUP(D31/$D$5,0)))</f>
+        <f>D31</f>
         <v>1</v>
       </c>
       <c r="F31" s="15" t="s">
@@ -3310,15 +3310,15 @@
       <c r="K31" s="15"/>
       <c r="L31" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F31,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G31,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H31,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I31,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J31,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K31,$A$11:$A$86,0)),0))</f>
-        <v>46366</v>
+        <v>46369</v>
       </c>
       <c r="M31" s="18">
         <f>IF(E31=0,IF(COUNTA(F31:K31)=0,$D$2,L31),WORKDAY.INTL(L31,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46369</v>
+        <v>46370</v>
       </c>
       <c r="N31" s="18">
         <f>IF(E31=0,M31,WORKDAY.INTL(M31,E31-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46369</v>
+        <v>46370</v>
       </c>
       <c r="O31" s="19"/>
       <c r="P31" s="15" t="s">
@@ -3356,15 +3356,15 @@
       <c r="K32" s="15"/>
       <c r="L32" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F32,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G32,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H32,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I32,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J32,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K32,$A$11:$A$86,0)),0))</f>
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="M32" s="18">
         <f>IF(E32=0,IF(COUNTA(F32:K32)=0,$D$2,L32),WORKDAY.INTL(L32,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="N32" s="18">
         <f>IF(E32=0,M32,WORKDAY.INTL(M32,E32-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="O32" s="19" t="s">
         <v>68</v>
@@ -3400,15 +3400,15 @@
       <c r="K33" s="15"/>
       <c r="L33" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F33,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G33,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H33,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I33,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J33,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K33,$A$11:$A$86,0)),0))</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="M33" s="18">
         <f>IF(E33=0,IF(COUNTA(F33:K33)=0,$D$2,L33),WORKDAY.INTL(L33,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46362</v>
+        <v>46363</v>
       </c>
       <c r="N33" s="18">
         <f>IF(E33=0,M33,WORKDAY.INTL(M33,E33-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46369</v>
+        <v>46370</v>
       </c>
       <c r="O33" s="19"/>
       <c r="P33" s="15" t="s">
@@ -3452,15 +3452,15 @@
       </c>
       <c r="L34" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F34,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G34,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H34,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I34,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J34,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K34,$A$11:$A$86,0)),0))</f>
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="M34" s="18">
         <f>IF(E34=0,IF(COUNTA(F34:K34)=0,$D$2,L34),WORKDAY.INTL(L34,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N34" s="18">
         <f>IF(E34=0,M34,WORKDAY.INTL(M34,E34-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46384</v>
+        <v>46385</v>
       </c>
       <c r="O34" s="19" t="s">
         <v>68</v>
@@ -3483,7 +3483,7 @@
         <v>2</v>
       </c>
       <c r="E35" s="15">
-        <f>IF(D35=0,0,MAX(1,ROUNDUP(D35/$D$5,0)))</f>
+        <f>D35</f>
         <v>2</v>
       </c>
       <c r="F35" s="15" t="s">
@@ -3496,15 +3496,15 @@
       <c r="K35" s="15"/>
       <c r="L35" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F35,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G35,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H35,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I35,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J35,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K35,$A$11:$A$86,0)),0))</f>
-        <v>46384</v>
+        <v>46385</v>
       </c>
       <c r="M35" s="18">
         <f>IF(E35=0,IF(COUNTA(F35:K35)=0,$D$2,L35),WORKDAY.INTL(L35,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N35" s="18">
         <f>IF(E35=0,M35,WORKDAY.INTL(M35,E35-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="O35" s="19" t="s">
         <v>68</v>
@@ -3630,15 +3630,15 @@
       <c r="K37" s="15"/>
       <c r="L37" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F37,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G37,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H37,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I37,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J37,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K37,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M37" s="18">
         <f>IF(E37=0,IF(COUNTA(F37:K37)=0,$D$2,L37),WORKDAY.INTL(L37,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N37" s="18">
         <f>IF(E37=0,M37,WORKDAY.INTL(M37,E37-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46399</v>
+        <v>46400</v>
       </c>
       <c r="O37" s="19"/>
       <c r="P37" s="15" t="s">
@@ -3674,15 +3674,15 @@
       <c r="K38" s="15"/>
       <c r="L38" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F38,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G38,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H38,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I38,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J38,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K38,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M38" s="18">
         <f>IF(E38=0,IF(COUNTA(F38:K38)=0,$D$2,L38),WORKDAY.INTL(L38,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N38" s="18">
         <f>IF(E38=0,M38,WORKDAY.INTL(M38,E38-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46405</v>
+        <v>46406</v>
       </c>
       <c r="O38" s="19"/>
       <c r="P38" s="15" t="s">
@@ -3716,15 +3716,15 @@
       <c r="K39" s="15"/>
       <c r="L39" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F39,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G39,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H39,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I39,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J39,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K39,$A$11:$A$86,0)),0))</f>
-        <v>46405</v>
+        <v>46406</v>
       </c>
       <c r="M39" s="18">
         <f>IF(E39=0,IF(COUNTA(F39:K39)=0,$D$2,L39),WORKDAY.INTL(L39,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46406</v>
+        <v>46407</v>
       </c>
       <c r="N39" s="18">
         <f>IF(E39=0,M39,WORKDAY.INTL(M39,E39-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46414</v>
+        <v>46415</v>
       </c>
       <c r="O39" s="19"/>
       <c r="P39" s="15" t="s">
@@ -3760,15 +3760,15 @@
       <c r="K40" s="15"/>
       <c r="L40" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F40,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G40,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H40,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I40,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J40,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K40,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M40" s="18">
         <f>IF(E40=0,IF(COUNTA(F40:K40)=0,$D$2,L40),WORKDAY.INTL(L40,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N40" s="18">
         <f>IF(E40=0,M40,WORKDAY.INTL(M40,E40-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="O40" s="19"/>
       <c r="P40" s="15" t="s">
@@ -3804,15 +3804,15 @@
       <c r="K41" s="15"/>
       <c r="L41" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F41,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G41,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H41,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I41,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J41,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K41,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M41" s="18">
         <f>IF(E41=0,IF(COUNTA(F41:K41)=0,$D$2,L41),WORKDAY.INTL(L41,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N41" s="18">
         <f>IF(E41=0,M41,WORKDAY.INTL(M41,E41-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="O41" s="19" t="s">
         <v>68</v>
@@ -3835,7 +3835,7 @@
         <v>2</v>
       </c>
       <c r="E42" s="15">
-        <f>IF(D42=0,0,MAX(1,ROUNDUP(D42/$D$5,0)))</f>
+        <f>D42</f>
         <v>2</v>
       </c>
       <c r="F42" s="15" t="s">
@@ -3856,15 +3856,15 @@
       <c r="K42" s="15"/>
       <c r="L42" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F42,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G42,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H42,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I42,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J42,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K42,$A$11:$A$86,0)),0))</f>
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="M42" s="18">
         <f>IF(E42=0,IF(COUNTA(F42:K42)=0,$D$2,L42),WORKDAY.INTL(L42,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46429</v>
+        <v>46432</v>
       </c>
       <c r="N42" s="18">
         <f>IF(E42=0,M42,WORKDAY.INTL(M42,E42-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46432</v>
+        <v>46433</v>
       </c>
       <c r="O42" s="19" t="s">
         <v>68</v>
@@ -3990,15 +3990,15 @@
       <c r="K44" s="15"/>
       <c r="L44" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F44,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G44,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H44,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I44,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J44,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K44,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M44" s="18">
         <f>IF(E44=0,IF(COUNTA(F44:K44)=0,$D$2,L44),WORKDAY.INTL(L44,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N44" s="18">
         <f>IF(E44=0,M44,WORKDAY.INTL(M44,E44-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="O44" s="19"/>
       <c r="P44" s="15" t="s">
@@ -4034,15 +4034,15 @@
       <c r="K45" s="15"/>
       <c r="L45" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F45,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G45,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H45,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I45,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J45,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K45,$A$11:$A$86,0)),0))</f>
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="M45" s="18">
         <f>IF(E45=0,IF(COUNTA(F45:K45)=0,$D$2,L45),WORKDAY.INTL(L45,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N45" s="18">
         <f>IF(E45=0,M45,WORKDAY.INTL(M45,E45-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46415</v>
+        <v>46418</v>
       </c>
       <c r="O45" s="19"/>
       <c r="P45" s="15" t="s">
@@ -4078,15 +4078,15 @@
       <c r="K46" s="15"/>
       <c r="L46" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F46,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G46,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H46,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I46,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J46,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K46,$A$11:$A$86,0)),0))</f>
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="M46" s="18">
         <f>IF(E46=0,IF(COUNTA(F46:K46)=0,$D$2,L46),WORKDAY.INTL(L46,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N46" s="18">
         <f>IF(E46=0,M46,WORKDAY.INTL(M46,E46-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46415</v>
+        <v>46418</v>
       </c>
       <c r="O46" s="19"/>
       <c r="P46" s="15" t="s">
@@ -4107,7 +4107,7 @@
         <v>3</v>
       </c>
       <c r="E47" s="15">
-        <f>IF(D47=0,0,MAX(1,ROUNDUP(D47/$D$5,0)))</f>
+        <f>D47</f>
         <v>3</v>
       </c>
       <c r="F47" s="15" t="s">
@@ -4120,15 +4120,15 @@
       <c r="K47" s="15"/>
       <c r="L47" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F47,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G47,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H47,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I47,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J47,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K47,$A$11:$A$86,0)),0))</f>
-        <v>46415</v>
+        <v>46418</v>
       </c>
       <c r="M47" s="18">
         <f>IF(E47=0,IF(COUNTA(F47:K47)=0,$D$2,L47),WORKDAY.INTL(L47,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46418</v>
+        <v>46419</v>
       </c>
       <c r="N47" s="18">
         <f>IF(E47=0,M47,WORKDAY.INTL(M47,E47-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="O47" s="19"/>
       <c r="P47" s="15" t="s">
@@ -4149,7 +4149,7 @@
         <v>3</v>
       </c>
       <c r="E48" s="15">
-        <f>IF(D48=0,0,MAX(1,ROUNDUP(D48/$D$5,0)))</f>
+        <f>D48</f>
         <v>3</v>
       </c>
       <c r="F48" s="15" t="s">
@@ -4162,15 +4162,15 @@
       <c r="K48" s="15"/>
       <c r="L48" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F48,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G48,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H48,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I48,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J48,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K48,$A$11:$A$86,0)),0))</f>
-        <v>46415</v>
+        <v>46418</v>
       </c>
       <c r="M48" s="18">
         <f>IF(E48=0,IF(COUNTA(F48:K48)=0,$D$2,L48),WORKDAY.INTL(L48,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46418</v>
+        <v>46419</v>
       </c>
       <c r="N48" s="18">
         <f>IF(E48=0,M48,WORKDAY.INTL(M48,E48-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="O48" s="19"/>
       <c r="P48" s="15" t="s">
@@ -4298,15 +4298,15 @@
       <c r="K50" s="15"/>
       <c r="L50" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F50,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G50,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H50,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I50,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J50,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K50,$A$11:$A$86,0)),0))</f>
-        <v>46432</v>
+        <v>46433</v>
       </c>
       <c r="M50" s="18">
         <f>IF(E50=0,IF(COUNTA(F50:K50)=0,$D$2,L50),WORKDAY.INTL(L50,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46433</v>
+        <v>46434</v>
       </c>
       <c r="N50" s="18">
         <f>IF(E50=0,M50,WORKDAY.INTL(M50,E50-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46447</v>
+        <v>46448</v>
       </c>
       <c r="O50" s="19" t="s">
         <v>68</v>
@@ -4342,15 +4342,15 @@
       <c r="K51" s="15"/>
       <c r="L51" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F51,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G51,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H51,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I51,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J51,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K51,$A$11:$A$86,0)),0))</f>
-        <v>46447</v>
+        <v>46448</v>
       </c>
       <c r="M51" s="18">
         <f>IF(E51=0,IF(COUNTA(F51:K51)=0,$D$2,L51),WORKDAY.INTL(L51,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46448</v>
+        <v>46449</v>
       </c>
       <c r="N51" s="18">
         <f>IF(E51=0,M51,WORKDAY.INTL(M51,E51-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46455</v>
+        <v>46456</v>
       </c>
       <c r="O51" s="19" t="s">
         <v>68</v>
@@ -4373,7 +4373,7 @@
         <v>2</v>
       </c>
       <c r="E52" s="15">
-        <f>IF(D52=0,0,MAX(1,ROUNDUP(D52/$D$5,0)))</f>
+        <f>D52</f>
         <v>2</v>
       </c>
       <c r="F52" s="15" t="s">
@@ -4386,15 +4386,15 @@
       <c r="K52" s="15"/>
       <c r="L52" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F52,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G52,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H52,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I52,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J52,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K52,$A$11:$A$86,0)),0))</f>
-        <v>46455</v>
+        <v>46456</v>
       </c>
       <c r="M52" s="18">
         <f>IF(E52=0,IF(COUNTA(F52:K52)=0,$D$2,L52),WORKDAY.INTL(L52,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46456</v>
+        <v>46457</v>
       </c>
       <c r="N52" s="18">
         <f>IF(E52=0,M52,WORKDAY.INTL(M52,E52-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46457</v>
+        <v>46460</v>
       </c>
       <c r="O52" s="19" t="s">
         <v>68</v>
@@ -4432,15 +4432,15 @@
       <c r="K53" s="15"/>
       <c r="L53" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F53,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G53,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H53,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I53,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J53,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K53,$A$11:$A$86,0)),0))</f>
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="M53" s="18">
         <f>IF(E53=0,IF(COUNTA(F53:K53)=0,$D$2,L53),WORKDAY.INTL(L53,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46421</v>
+        <v>46422</v>
       </c>
       <c r="N53" s="18">
         <f>IF(E53=0,M53,WORKDAY.INTL(M53,E53-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="O53" s="19"/>
       <c r="P53" s="15" t="s">
@@ -4476,15 +4476,15 @@
       <c r="K54" s="15"/>
       <c r="L54" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F54,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G54,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H54,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I54,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J54,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K54,$A$11:$A$86,0)),0))</f>
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="M54" s="18">
         <f>IF(E54=0,IF(COUNTA(F54:K54)=0,$D$2,L54),WORKDAY.INTL(L54,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46421</v>
+        <v>46422</v>
       </c>
       <c r="N54" s="18">
         <f>IF(E54=0,M54,WORKDAY.INTL(M54,E54-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="O54" s="19"/>
       <c r="P54" s="15" t="s">
@@ -4505,7 +4505,7 @@
         <v>3</v>
       </c>
       <c r="E55" s="15">
-        <f>IF(D55=0,0,MAX(1,ROUNDUP(D55/$D$5,0)))</f>
+        <f>D55</f>
         <v>3</v>
       </c>
       <c r="F55" s="15" t="s">
@@ -4520,15 +4520,15 @@
       <c r="K55" s="15"/>
       <c r="L55" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F55,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G55,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H55,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I55,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J55,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K55,$A$11:$A$86,0)),0))</f>
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="M55" s="18">
         <f>IF(E55=0,IF(COUNTA(F55:K55)=0,$D$2,L55),WORKDAY.INTL(L55,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46429</v>
+        <v>46432</v>
       </c>
       <c r="N55" s="18">
         <f>IF(E55=0,M55,WORKDAY.INTL(M55,E55-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46433</v>
+        <v>46434</v>
       </c>
       <c r="O55" s="19"/>
       <c r="P55" s="15" t="s">
@@ -4549,7 +4549,7 @@
         <v>1</v>
       </c>
       <c r="E56" s="15">
-        <f>IF(D56=0,0,MAX(1,ROUNDUP(D56/$D$5,0)))</f>
+        <f>D56</f>
         <v>1</v>
       </c>
       <c r="F56" s="15" t="s">
@@ -4562,15 +4562,15 @@
       <c r="K56" s="15"/>
       <c r="L56" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F56,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G56,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H56,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I56,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J56,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K56,$A$11:$A$86,0)),0))</f>
-        <v>46433</v>
+        <v>46434</v>
       </c>
       <c r="M56" s="18">
         <f>IF(E56=0,IF(COUNTA(F56:K56)=0,$D$2,L56),WORKDAY.INTL(L56,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46434</v>
+        <v>46435</v>
       </c>
       <c r="N56" s="18">
         <f>IF(E56=0,M56,WORKDAY.INTL(M56,E56-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46434</v>
+        <v>46435</v>
       </c>
       <c r="O56" s="19"/>
       <c r="P56" s="15" t="s">
@@ -4681,8 +4681,8 @@
         <v>40</v>
       </c>
       <c r="E58" s="15">
-        <f>IF(D58=0,0,MAX(1,ROUNDUP(D58/$D$5,0)))</f>
-        <v>34</v>
+        <f>D58</f>
+        <v>40</v>
       </c>
       <c r="F58" s="15" t="s">
         <v>130</v>
@@ -4694,15 +4694,15 @@
       <c r="K58" s="15"/>
       <c r="L58" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F58,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G58,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H58,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I58,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J58,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K58,$A$11:$A$86,0)),0))</f>
-        <v>46386</v>
+        <v>46387</v>
       </c>
       <c r="M58" s="18">
         <f>IF(E58=0,IF(COUNTA(F58:K58)=0,$D$2,L58),WORKDAY.INTL(L58,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46390</v>
       </c>
       <c r="N58" s="18">
         <f>IF(E58=0,M58,WORKDAY.INTL(M58,E58-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46434</v>
+        <v>46443</v>
       </c>
       <c r="O58" s="19"/>
       <c r="P58" s="15" t="s">
@@ -4740,15 +4740,15 @@
       <c r="K59" s="15"/>
       <c r="L59" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F59,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G59,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H59,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I59,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J59,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K59,$A$11:$A$86,0)),0))</f>
-        <v>46434</v>
+        <v>46443</v>
       </c>
       <c r="M59" s="18">
         <f>IF(E59=0,IF(COUNTA(F59:K59)=0,$D$2,L59),WORKDAY.INTL(L59,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46435</v>
+        <v>46446</v>
       </c>
       <c r="N59" s="18">
         <f>IF(E59=0,M59,WORKDAY.INTL(M59,E59-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46457</v>
+        <v>46468</v>
       </c>
       <c r="O59" s="19"/>
       <c r="P59" s="15" t="s">
@@ -4784,15 +4784,15 @@
       <c r="K60" s="15"/>
       <c r="L60" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F60,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G60,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H60,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I60,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J60,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K60,$A$11:$A$86,0)),0))</f>
-        <v>46457</v>
+        <v>46468</v>
       </c>
       <c r="M60" s="18">
         <f>IF(E60=0,IF(COUNTA(F60:K60)=0,$D$2,L60),WORKDAY.INTL(L60,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46460</v>
+        <v>46469</v>
       </c>
       <c r="N60" s="18">
         <f>IF(E60=0,M60,WORKDAY.INTL(M60,E60-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46468</v>
+        <v>46477</v>
       </c>
       <c r="O60" s="19"/>
       <c r="P60" s="15" t="s">
@@ -4828,15 +4828,15 @@
       <c r="K61" s="15"/>
       <c r="L61" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F61,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G61,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H61,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I61,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J61,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K61,$A$11:$A$86,0)),0))</f>
-        <v>46468</v>
+        <v>46477</v>
       </c>
       <c r="M61" s="18">
         <f>IF(E61=0,IF(COUNTA(F61:K61)=0,$D$2,L61),WORKDAY.INTL(L61,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46469</v>
+        <v>46478</v>
       </c>
       <c r="N61" s="18">
         <f>IF(E61=0,M61,WORKDAY.INTL(M61,E61-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46474</v>
+        <v>46483</v>
       </c>
       <c r="O61" s="19"/>
       <c r="P61" s="15" t="s">
@@ -4962,15 +4962,15 @@
       <c r="K63" s="15"/>
       <c r="L63" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F63,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G63,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H63,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I63,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J63,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K63,$A$11:$A$86,0)),0))</f>
-        <v>46457</v>
+        <v>46460</v>
       </c>
       <c r="M63" s="18">
         <f>IF(E63=0,IF(COUNTA(F63:K63)=0,$D$2,L63),WORKDAY.INTL(L63,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46460</v>
+        <v>46461</v>
       </c>
       <c r="N63" s="18">
         <f>IF(E63=0,M63,WORKDAY.INTL(M63,E63-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46474</v>
+        <v>46475</v>
       </c>
       <c r="O63" s="19"/>
       <c r="P63" s="15" t="s">
@@ -5008,15 +5008,15 @@
       <c r="K64" s="15"/>
       <c r="L64" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F64,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G64,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H64,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I64,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J64,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K64,$A$11:$A$86,0)),0))</f>
-        <v>46457</v>
+        <v>46460</v>
       </c>
       <c r="M64" s="18">
         <f>IF(E64=0,IF(COUNTA(F64:K64)=0,$D$2,L64),WORKDAY.INTL(L64,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46460</v>
+        <v>46461</v>
       </c>
       <c r="N64" s="18">
         <f>IF(E64=0,M64,WORKDAY.INTL(M64,E64-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46475</v>
+        <v>46476</v>
       </c>
       <c r="O64" s="19" t="s">
         <v>68</v>
@@ -5054,15 +5054,15 @@
       <c r="K65" s="15"/>
       <c r="L65" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F65,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G65,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H65,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I65,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J65,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K65,$A$11:$A$86,0)),0))</f>
-        <v>46434</v>
+        <v>46435</v>
       </c>
       <c r="M65" s="18">
         <f>IF(E65=0,IF(COUNTA(F65:K65)=0,$D$2,L65),WORKDAY.INTL(L65,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46435</v>
+        <v>46436</v>
       </c>
       <c r="N65" s="18">
         <f>IF(E65=0,M65,WORKDAY.INTL(M65,E65-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46443</v>
+        <v>46446</v>
       </c>
       <c r="O65" s="19"/>
       <c r="P65" s="15" t="s">
@@ -5098,15 +5098,15 @@
       <c r="K66" s="15"/>
       <c r="L66" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F66,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G66,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H66,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I66,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J66,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K66,$A$11:$A$86,0)),0))</f>
-        <v>46433</v>
+        <v>46434</v>
       </c>
       <c r="M66" s="18">
         <f>IF(E66=0,IF(COUNTA(F66:K66)=0,$D$2,L66),WORKDAY.INTL(L66,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46434</v>
+        <v>46435</v>
       </c>
       <c r="N66" s="18">
         <f>IF(E66=0,M66,WORKDAY.INTL(M66,E66-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46453</v>
+        <v>46454</v>
       </c>
       <c r="O66" s="19"/>
       <c r="P66" s="15" t="s">
@@ -5146,15 +5146,15 @@
       <c r="K67" s="15"/>
       <c r="L67" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F67,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G67,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H67,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I67,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J67,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K67,$A$11:$A$86,0)),0))</f>
-        <v>46475</v>
+        <v>46476</v>
       </c>
       <c r="M67" s="18">
         <f>IF(E67=0,IF(COUNTA(F67:K67)=0,$D$2,L67),WORKDAY.INTL(L67,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46476</v>
+        <v>46477</v>
       </c>
       <c r="N67" s="18">
         <f>IF(E67=0,M67,WORKDAY.INTL(M67,E67-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46484</v>
+        <v>46485</v>
       </c>
       <c r="O67" s="19"/>
       <c r="P67" s="15" t="s">
@@ -5192,15 +5192,15 @@
       <c r="K68" s="15"/>
       <c r="L68" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F68,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G68,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H68,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I68,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J68,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K68,$A$11:$A$86,0)),0))</f>
-        <v>46475</v>
+        <v>46476</v>
       </c>
       <c r="M68" s="18">
         <f>IF(E68=0,IF(COUNTA(F68:K68)=0,$D$2,L68),WORKDAY.INTL(L68,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46476</v>
+        <v>46477</v>
       </c>
       <c r="N68" s="18">
         <f>IF(E68=0,M68,WORKDAY.INTL(M68,E68-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46490</v>
+        <v>46491</v>
       </c>
       <c r="O68" s="19" t="s">
         <v>68</v>
@@ -5242,15 +5242,15 @@
       <c r="K69" s="15"/>
       <c r="L69" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F69,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G69,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H69,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I69,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J69,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K69,$A$11:$A$86,0)),0))</f>
-        <v>46490</v>
+        <v>46491</v>
       </c>
       <c r="M69" s="18">
         <f>IF(E69=0,IF(COUNTA(F69:K69)=0,$D$2,L69),WORKDAY.INTL(L69,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46491</v>
+        <v>46492</v>
       </c>
       <c r="N69" s="18">
         <f>IF(E69=0,M69,WORKDAY.INTL(M69,E69-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46516</v>
+        <v>46517</v>
       </c>
       <c r="O69" s="19" t="s">
         <v>68</v>
@@ -5286,15 +5286,15 @@
       <c r="K70" s="15"/>
       <c r="L70" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F70,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G70,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H70,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I70,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J70,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K70,$A$11:$A$86,0)),0))</f>
-        <v>46516</v>
+        <v>46517</v>
       </c>
       <c r="M70" s="18">
         <f>IF(E70=0,IF(COUNTA(F70:K70)=0,$D$2,L70),WORKDAY.INTL(L70,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46517</v>
+        <v>46518</v>
       </c>
       <c r="N70" s="18">
         <f>IF(E70=0,M70,WORKDAY.INTL(M70,E70-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46526</v>
+        <v>46527</v>
       </c>
       <c r="O70" s="19"/>
       <c r="P70" s="15" t="s">
@@ -5328,15 +5328,15 @@
       <c r="K71" s="15"/>
       <c r="L71" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F71,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G71,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H71,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I71,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J71,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K71,$A$11:$A$86,0)),0))</f>
-        <v>46516</v>
+        <v>46517</v>
       </c>
       <c r="M71" s="18">
         <f>IF(E71=0,IF(COUNTA(F71:K71)=0,$D$2,L71),WORKDAY.INTL(L71,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46517</v>
+        <v>46518</v>
       </c>
       <c r="N71" s="18">
         <f>IF(E71=0,M71,WORKDAY.INTL(M71,E71-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46520</v>
+        <v>46523</v>
       </c>
       <c r="O71" s="19"/>
       <c r="P71" s="15" t="s">
@@ -5374,15 +5374,15 @@
       <c r="K72" s="15"/>
       <c r="L72" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F72,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G72,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H72,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I72,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J72,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K72,$A$11:$A$86,0)),0))</f>
-        <v>46516</v>
+        <v>46517</v>
       </c>
       <c r="M72" s="18">
         <f>IF(E72=0,IF(COUNTA(F72:K72)=0,$D$2,L72),WORKDAY.INTL(L72,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46517</v>
+        <v>46518</v>
       </c>
       <c r="N72" s="18">
         <f>IF(E72=0,M72,WORKDAY.INTL(M72,E72-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46526</v>
+        <v>46527</v>
       </c>
       <c r="O72" s="19" t="s">
         <v>68</v>
@@ -5510,15 +5510,15 @@
       <c r="K74" s="15"/>
       <c r="L74" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F74,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G74,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H74,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I74,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J74,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K74,$A$11:$A$86,0)),0))</f>
-        <v>46380</v>
+        <v>46390</v>
       </c>
       <c r="M74" s="18">
         <f>IF(E74=0,IF(COUNTA(F74:K74)=0,$D$2,L74),WORKDAY.INTL(L74,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46383</v>
+        <v>46391</v>
       </c>
       <c r="N74" s="18">
         <f>IF(E74=0,M74,WORKDAY.INTL(M74,E74-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46387</v>
+        <v>46397</v>
       </c>
       <c r="O74" s="19"/>
       <c r="P74" s="15" t="s">
@@ -5552,15 +5552,15 @@
       <c r="K75" s="15"/>
       <c r="L75" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F75,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G75,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H75,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I75,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J75,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K75,$A$11:$A$86,0)),0))</f>
-        <v>46457</v>
+        <v>46468</v>
       </c>
       <c r="M75" s="18">
         <f>IF(E75=0,IF(COUNTA(F75:K75)=0,$D$2,L75),WORKDAY.INTL(L75,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46460</v>
+        <v>46469</v>
       </c>
       <c r="N75" s="18">
         <f>IF(E75=0,M75,WORKDAY.INTL(M75,E75-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46469</v>
+        <v>46478</v>
       </c>
       <c r="O75" s="19"/>
       <c r="P75" s="15" t="s">
@@ -5594,15 +5594,15 @@
       <c r="K76" s="15"/>
       <c r="L76" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F76,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G76,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H76,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I76,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J76,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K76,$A$11:$A$86,0)),0))</f>
-        <v>46469</v>
+        <v>46478</v>
       </c>
       <c r="M76" s="18">
         <f>IF(E76=0,IF(COUNTA(F76:K76)=0,$D$2,L76),WORKDAY.INTL(L76,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46470</v>
+        <v>46481</v>
       </c>
       <c r="N76" s="18">
         <f>IF(E76=0,M76,WORKDAY.INTL(M76,E76-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46477</v>
+        <v>46488</v>
       </c>
       <c r="O76" s="19"/>
       <c r="P76" s="15" t="s">
@@ -5638,15 +5638,15 @@
       <c r="K77" s="15"/>
       <c r="L77" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F77,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G77,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H77,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I77,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J77,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K77,$A$11:$A$86,0)),0))</f>
-        <v>46477</v>
+        <v>46488</v>
       </c>
       <c r="M77" s="18">
         <f>IF(E77=0,IF(COUNTA(F77:K77)=0,$D$2,L77),WORKDAY.INTL(L77,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46478</v>
+        <v>46489</v>
       </c>
       <c r="N77" s="18">
         <f>IF(E77=0,M77,WORKDAY.INTL(M77,E77-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46491</v>
+        <v>46509</v>
       </c>
       <c r="O77" s="19"/>
       <c r="P77" s="15" t="s">
@@ -5776,15 +5776,15 @@
       <c r="K79" s="15"/>
       <c r="L79" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F79,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G79,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H79,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I79,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J79,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K79,$A$11:$A$86,0)),0))</f>
-        <v>46526</v>
+        <v>46527</v>
       </c>
       <c r="M79" s="18">
         <f>IF(E79=0,IF(COUNTA(F79:K79)=0,$D$2,L79),WORKDAY.INTL(L79,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46527</v>
+        <v>46530</v>
       </c>
       <c r="N79" s="18">
         <f>IF(E79=0,M79,WORKDAY.INTL(M79,E79-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46531</v>
+        <v>46532</v>
       </c>
       <c r="O79" s="19"/>
       <c r="P79" s="15" t="s">
@@ -5818,15 +5818,15 @@
       <c r="K80" s="15"/>
       <c r="L80" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F80,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G80,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H80,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I80,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J80,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K80,$A$11:$A$86,0)),0))</f>
-        <v>46526</v>
+        <v>46527</v>
       </c>
       <c r="M80" s="18">
         <f>IF(E80=0,IF(COUNTA(F80:K80)=0,$D$2,L80),WORKDAY.INTL(L80,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46527</v>
+        <v>46530</v>
       </c>
       <c r="N80" s="18">
         <f>IF(E80=0,M80,WORKDAY.INTL(M80,E80-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46532</v>
+        <v>46533</v>
       </c>
       <c r="O80" s="19" t="s">
         <v>68</v>
@@ -5870,15 +5870,15 @@
       <c r="K81" s="15"/>
       <c r="L81" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F81,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G81,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H81,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I81,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J81,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K81,$A$11:$A$86,0)),0))</f>
-        <v>46526</v>
+        <v>46527</v>
       </c>
       <c r="M81" s="18">
         <f>IF(E81=0,IF(COUNTA(F81:K81)=0,$D$2,L81),WORKDAY.INTL(L81,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46527</v>
+        <v>46530</v>
       </c>
       <c r="N81" s="18">
         <f>IF(E81=0,M81,WORKDAY.INTL(M81,E81-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46531</v>
+        <v>46532</v>
       </c>
       <c r="O81" s="19"/>
       <c r="P81" s="15" t="s">
@@ -5899,7 +5899,7 @@
         <v>3</v>
       </c>
       <c r="E82" s="15">
-        <f>IF(D82=0,0,MAX(1,ROUNDUP(D82/$D$5,0)))</f>
+        <f>D82</f>
         <v>3</v>
       </c>
       <c r="F82" s="15" t="s">
@@ -5916,15 +5916,15 @@
       <c r="K82" s="15"/>
       <c r="L82" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F82,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G82,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H82,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I82,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J82,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K82,$A$11:$A$86,0)),0))</f>
-        <v>46532</v>
+        <v>46533</v>
       </c>
       <c r="M82" s="18">
         <f>IF(E82=0,IF(COUNTA(F82:K82)=0,$D$2,L82),WORKDAY.INTL(L82,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46533</v>
+        <v>46534</v>
       </c>
       <c r="N82" s="18">
         <f>IF(E82=0,M82,WORKDAY.INTL(M82,E82-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46537</v>
+        <v>46538</v>
       </c>
       <c r="O82" s="19" t="s">
         <v>68</v>
@@ -5960,15 +5960,15 @@
       <c r="K83" s="15"/>
       <c r="L83" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F83,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G83,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H83,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I83,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J83,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K83,$A$11:$A$86,0)),0))</f>
-        <v>46537</v>
+        <v>46538</v>
       </c>
       <c r="M83" s="18">
         <f>IF(E83=0,IF(COUNTA(F83:K83)=0,$D$2,L83),WORKDAY.INTL(L83,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46538</v>
+        <v>46539</v>
       </c>
       <c r="N83" s="18">
         <f>IF(E83=0,M83,WORKDAY.INTL(M83,E83-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46546</v>
+        <v>46547</v>
       </c>
       <c r="O83" s="19"/>
       <c r="P83" s="15" t="s">
@@ -5989,8 +5989,8 @@
         <v>10</v>
       </c>
       <c r="E84" s="15">
-        <f>IF(D84=0,0,MAX(1,ROUNDUP(D84/$D$5,0)))</f>
-        <v>9</v>
+        <f>D84</f>
+        <v>10</v>
       </c>
       <c r="F84" s="15" t="s">
         <v>247</v>
@@ -6002,15 +6002,15 @@
       <c r="K84" s="15"/>
       <c r="L84" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F84,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G84,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H84,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I84,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J84,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K84,$A$11:$A$86,0)),0))</f>
-        <v>46537</v>
+        <v>46538</v>
       </c>
       <c r="M84" s="18">
         <f>IF(E84=0,IF(COUNTA(F84:K84)=0,$D$2,L84),WORKDAY.INTL(L84,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46538</v>
+        <v>46539</v>
       </c>
       <c r="N84" s="18">
         <f>IF(E84=0,M84,WORKDAY.INTL(M84,E84-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46548</v>
+        <v>46552</v>
       </c>
       <c r="O84" s="19" t="s">
         <v>68</v>
@@ -6046,15 +6046,15 @@
       <c r="K85" s="15"/>
       <c r="L85" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F85,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G85,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H85,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I85,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J85,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K85,$A$11:$A$86,0)),0))</f>
-        <v>46546</v>
+        <v>46547</v>
       </c>
       <c r="M85" s="18">
         <f>IF(E85=0,IF(COUNTA(F85:K85)=0,$D$2,L85),WORKDAY.INTL(L85,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46546</v>
+        <v>46547</v>
       </c>
       <c r="N85" s="18">
         <f>IF(E85=0,M85,WORKDAY.INTL(M85,E85-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46546</v>
+        <v>46547</v>
       </c>
       <c r="O85" s="19"/>
       <c r="P85" s="15" t="s">
@@ -6075,8 +6075,8 @@
         <v>30</v>
       </c>
       <c r="E86" s="15">
-        <f>IF(D86=0,0,MAX(1,ROUNDUP(D86/$D$5,0)))</f>
-        <v>26</v>
+        <f>D86</f>
+        <v>30</v>
       </c>
       <c r="F86" s="15" t="s">
         <v>251</v>
@@ -6090,15 +6090,15 @@
       <c r="K86" s="15"/>
       <c r="L86" s="18">
         <f>MAX($D$2-1,IFERROR(INDEX($N$11:$N$86,MATCH(F86,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(G86,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(H86,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(I86,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(J86,$A$11:$A$86,0)),0),IFERROR(INDEX($N$11:$N$86,MATCH(K86,$A$11:$A$86,0)),0))</f>
-        <v>46548</v>
+        <v>46552</v>
       </c>
       <c r="M86" s="18">
         <f>IF(E86=0,IF(COUNTA(F86:K86)=0,$D$2,L86),WORKDAY.INTL(L86,1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46551</v>
+        <v>46553</v>
       </c>
       <c r="N86" s="18">
         <f>IF(E86=0,M86,WORKDAY.INTL(M86,E86-1,$D$3,'לוח שנה וחגים'!$F$5:$F$20))</f>
-        <v>46586</v>
+        <v>46594</v>
       </c>
       <c r="O86" s="19"/>
       <c r="P86" s="15" t="s">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="N88" s="20">
         <f>N85</f>
-        <v>46546</v>
+        <v>46547</v>
       </c>
     </row>
     <row r="89" spans="1:16">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="N89" s="20">
         <f>N86</f>
-        <v>46586</v>
+        <v>46594</v>
       </c>
     </row>
     <row r="90" spans="1:16">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="N90" s="21">
         <f>ROUND((N88-$D$2+1)/7,1)</f>
-        <v>30.4</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="91" spans="1:16">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="N91" s="21">
         <f>NETWORKDAYS.INTL($D$2,N88,$D$3,'לוח שנה וחגים'!$F$5:$F$20)</f>
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="92" spans="1:16">

</xml_diff>